<commit_message>
Updated Files (Delete OLD Ribbon PCB File from Repo)
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/Control-Board/LCSC_BOM-Control-Board.xlsx
+++ b/Deliverables/BOM/Control-Board/LCSC_BOM-Control-Board.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\ManarHarake-sEMGDevice\Deliverables\BOM\Control-Board\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD8D14E0-9850-4399-8944-24ACDF90D335}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97468936-EFA4-47EE-9780-6796292DE8E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="840" windowWidth="11790" windowHeight="15360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-5700" yWindow="3960" windowWidth="11790" windowHeight="15360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t>#</t>
   </si>
@@ -72,9 +72,6 @@
   </si>
   <si>
     <t>C498674</t>
-  </si>
-  <si>
-    <t>C158011</t>
   </si>
   <si>
     <t>C557729</t>
@@ -660,7 +657,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9C0EAC8-2749-4D8B-AD6B-98E76B44D0B5}">
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
@@ -805,76 +802,76 @@
       <c r="A14" s="10">
         <v>12</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C14" s="2">
-        <v>20</v>
+      <c r="C14" s="1">
+        <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="10">
         <v>13</v>
       </c>
-      <c r="B15" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C15" s="1">
-        <v>6</v>
+      <c r="B15" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C15" s="2">
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="10">
         <v>14</v>
       </c>
-      <c r="B16" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="C16" s="2">
-        <v>10</v>
+      <c r="B16" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C16" s="1">
+        <v>6</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="10">
         <v>15</v>
       </c>
-      <c r="B17" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="C17" s="1">
-        <v>6</v>
+      <c r="B17" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C17" s="2">
+        <v>20</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="10">
         <v>16</v>
       </c>
-      <c r="B18" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="C18" s="2">
-        <v>20</v>
+      <c r="B18" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="5">
+        <v>7</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="10">
         <v>17</v>
       </c>
-      <c r="B19" s="9" t="s">
+      <c r="B19" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C19" s="5">
-        <v>7</v>
+      <c r="C19" s="2">
+        <v>10</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="10">
         <v>18</v>
       </c>
-      <c r="B20" s="8" t="s">
+      <c r="B20" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C20" s="2">
+      <c r="C20" s="5">
         <v>10</v>
       </c>
     </row>
@@ -882,10 +879,10 @@
       <c r="A21" s="10">
         <v>19</v>
       </c>
-      <c r="B21" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="C21" s="5">
+      <c r="B21" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C21" s="2">
         <v>10</v>
       </c>
     </row>
@@ -893,76 +890,76 @@
       <c r="A22" s="10">
         <v>20</v>
       </c>
-      <c r="B22" s="8" t="s">
+      <c r="B22" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C22" s="2">
-        <v>10</v>
+      <c r="C22" s="5">
+        <v>50</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="10">
         <v>21</v>
       </c>
-      <c r="B23" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="C23" s="5">
-        <v>50</v>
+      <c r="B23" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C23" s="2">
+        <v>10</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="10">
         <v>22</v>
       </c>
-      <c r="B24" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="C24" s="2">
-        <v>10</v>
+      <c r="B24" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C24" s="5">
+        <v>50</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="10">
         <v>23</v>
       </c>
-      <c r="B25" s="9" t="s">
+      <c r="B25" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="C25" s="5">
-        <v>50</v>
+      <c r="C25" s="2">
+        <v>10</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="10">
         <v>24</v>
       </c>
-      <c r="B26" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="C26" s="2">
-        <v>10</v>
+      <c r="B26" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="C26" s="5">
+        <v>50</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="10">
         <v>25</v>
       </c>
-      <c r="B27" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="C27" s="5">
-        <v>50</v>
+      <c r="B27" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C27" s="2">
+        <v>100</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="10">
         <v>26</v>
       </c>
-      <c r="B28" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="C28" s="2">
+      <c r="B28" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C28" s="5">
         <v>100</v>
       </c>
     </row>
@@ -970,10 +967,10 @@
       <c r="A29" s="10">
         <v>27</v>
       </c>
-      <c r="B29" s="9" t="s">
+      <c r="B29" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="C29" s="5">
+      <c r="C29" s="2">
         <v>100</v>
       </c>
     </row>
@@ -981,10 +978,10 @@
       <c r="A30" s="10">
         <v>28</v>
       </c>
-      <c r="B30" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="C30" s="2">
+      <c r="B30" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C30" s="5">
         <v>100</v>
       </c>
     </row>
@@ -992,10 +989,10 @@
       <c r="A31" s="10">
         <v>29</v>
       </c>
-      <c r="B31" s="9" t="s">
+      <c r="B31" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="C31" s="5">
+      <c r="C31" s="2">
         <v>100</v>
       </c>
     </row>
@@ -1003,10 +1000,10 @@
       <c r="A32" s="10">
         <v>30</v>
       </c>
-      <c r="B32" s="8" t="s">
+      <c r="B32" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="C32" s="2">
+      <c r="C32" s="5">
         <v>100</v>
       </c>
     </row>
@@ -1014,43 +1011,43 @@
       <c r="A33" s="10">
         <v>31</v>
       </c>
-      <c r="B33" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="C33" s="5">
-        <v>100</v>
+      <c r="B33" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="C33" s="2">
+        <v>50</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="10">
         <v>32</v>
       </c>
-      <c r="B34" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="C34" s="2">
-        <v>50</v>
+      <c r="B34" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C34" s="5">
+        <v>10</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="10">
         <v>33</v>
       </c>
-      <c r="B35" s="9" t="s">
+      <c r="B35" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="C35" s="5">
-        <v>10</v>
+      <c r="C35" s="2">
+        <v>6</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="10">
         <v>34</v>
       </c>
-      <c r="B36" s="8" t="s">
+      <c r="B36" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="C36" s="2">
+      <c r="C36" s="5">
         <v>6</v>
       </c>
     </row>
@@ -1058,10 +1055,10 @@
       <c r="A37" s="10">
         <v>35</v>
       </c>
-      <c r="B37" s="9" t="s">
+      <c r="B37" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="C37" s="5">
+      <c r="C37" s="2">
         <v>6</v>
       </c>
     </row>
@@ -1069,10 +1066,10 @@
       <c r="A38" s="10">
         <v>36</v>
       </c>
-      <c r="B38" s="8" t="s">
+      <c r="B38" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="C38" s="2">
+      <c r="C38" s="5">
         <v>6</v>
       </c>
     </row>
@@ -1080,54 +1077,43 @@
       <c r="A39" s="10">
         <v>37</v>
       </c>
-      <c r="B39" s="9" t="s">
+      <c r="B39" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="C39" s="5">
-        <v>6</v>
+      <c r="C39" s="2">
+        <v>10</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="10">
         <v>38</v>
       </c>
-      <c r="B40" s="8" t="s">
+      <c r="B40" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="C40" s="2">
-        <v>10</v>
+      <c r="C40" s="5">
+        <v>11</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="10">
         <v>39</v>
       </c>
-      <c r="B41" s="9" t="s">
+      <c r="B41" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="C41" s="5">
-        <v>11</v>
+      <c r="C41" s="2">
+        <v>10</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="10">
         <v>40</v>
       </c>
-      <c r="B42" s="8" t="s">
+      <c r="B42" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="C42" s="2">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="10">
-        <v>41</v>
-      </c>
-      <c r="B43" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="C43" s="12">
+      <c r="C42" s="12">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
S.No 3 incorrect entry corrected in Control Board BOM
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/Control-Board/LCSC_BOM-Control-Board.xlsx
+++ b/Deliverables/BOM/Control-Board/LCSC_BOM-Control-Board.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25225"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25501"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\ManarHarake-sEMGDevice\Deliverables\BOM\Control-Board\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\ManarHarake-sEMGDevice\Deliverables\BOM\Control-Board\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97468936-EFA4-47EE-9780-6796292DE8E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9D74F65-DB6C-4ED4-B9ED-0A597398DB3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-5700" yWindow="3960" windowWidth="11790" windowHeight="15360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -47,9 +47,6 @@
     <t>C307331</t>
   </si>
   <si>
-    <t>C2922482</t>
-  </si>
-  <si>
     <t>C412302</t>
   </si>
   <si>
@@ -159,6 +156,9 @@
   </si>
   <si>
     <t>C620515</t>
+  </si>
+  <si>
+    <t>C91606</t>
   </si>
 </sst>
 </file>
@@ -658,15 +658,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9C0EAC8-2749-4D8B-AD6B-98E76B44D0B5}">
   <dimension ref="A1:C42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
@@ -677,7 +677,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="10">
         <v>1</v>
       </c>
@@ -688,7 +688,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="10">
         <v>2</v>
       </c>
@@ -699,419 +699,419 @@
         <v>150</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="10">
         <v>3</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>5</v>
+        <v>42</v>
       </c>
       <c r="C5" s="1">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="10">
         <v>4</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C6" s="2">
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="10">
         <v>5</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C7" s="1">
         <v>50</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="10">
         <v>6</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C8" s="2">
         <v>50</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="10">
         <v>7</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C9" s="5">
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="10">
         <v>8</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C10" s="2">
         <v>100</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="10">
         <v>9</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C11" s="1">
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="10">
         <v>10</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C12" s="2">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="10">
         <v>11</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C13" s="1">
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="10">
         <v>12</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C14" s="1">
         <v>6</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="10">
         <v>13</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C15" s="2">
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="10">
         <v>14</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C16" s="1">
         <v>6</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="10">
         <v>15</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C17" s="2">
         <v>20</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="10">
         <v>16</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C18" s="5">
         <v>7</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="10">
         <v>17</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C19" s="2">
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="10">
         <v>18</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C20" s="5">
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="10">
         <v>19</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C21" s="2">
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="10">
         <v>20</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C22" s="5">
         <v>50</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="10">
         <v>21</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C23" s="2">
         <v>10</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="10">
         <v>22</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C24" s="5">
         <v>50</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="10">
         <v>23</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C25" s="2">
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="10">
         <v>24</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C26" s="5">
         <v>50</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="10">
         <v>25</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C27" s="2">
         <v>100</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="10">
         <v>26</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C28" s="5">
         <v>100</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="10">
         <v>27</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C29" s="2">
         <v>100</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="10">
         <v>28</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C30" s="5">
         <v>100</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="10">
         <v>29</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C31" s="2">
         <v>100</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="10">
         <v>30</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C32" s="5">
         <v>100</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A33" s="10">
         <v>31</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C33" s="2">
         <v>50</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A34" s="10">
         <v>32</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C34" s="5">
         <v>10</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="10">
         <v>33</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C35" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="36" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A36" s="10">
         <v>34</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C36" s="5">
         <v>6</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A37" s="10">
         <v>35</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C37" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="38" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A38" s="10">
         <v>36</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C38" s="5">
         <v>6</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A39" s="10">
         <v>37</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C39" s="2">
         <v>10</v>
       </c>
     </row>
-    <row r="40" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A40" s="10">
         <v>38</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C40" s="5">
         <v>11</v>
       </c>
     </row>
-    <row r="41" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A41" s="10">
         <v>39</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C41" s="2">
         <v>10</v>
       </c>
     </row>
-    <row r="42" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A42" s="10">
         <v>40</v>
       </c>
       <c r="B42" s="11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C42" s="12">
         <v>10</v>

</xml_diff>